<commit_message>
Validate balance evidence and integrate the frozen worth campaign
Resolve the approved source conflicts and repair calibration, criterion scope,
provenance, completion and workbook checks. Import only complete campaign data
with checked source, specs, schedules and raw hashes; keep price adoption separate.

Record the reviewed reports and active campaign handoff. The full test suite,
artwork checks and strict balance audit pass. No game rules or prices change.

Co-Authored-By: Codex <noreply@openai.com>
</commit_message>
<xml_diff>
--- a/docs/status/king-down-status-2026-10-09.xlsx
+++ b/docs/status/king-down-status-2026-10-09.xlsx
@@ -1789,7 +1789,7 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Each side gets the same six random one-use cards from the deal.</t>
+          <t>Each side starts with the same four random one-use cards from the deal.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
@@ -4457,12 +4457,12 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>The king plus 7 pieces drawn from QORRBBNNAAGMMS, in the same order for both sides.</t>
+          <t>The back rank is drawn from QOLRRBBNNAAGMMS, with one Paladin in the pool.</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>Paladin out, ogre in (2026-09-24). One beast per army (2026-10-04). Owner 2026-10-09: Paladin back in the pool next to the Ogre (being built).</t>
+          <t>Current pool: src/rules/setup.ts POOL. Paladin and Ogre are built.</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
@@ -4525,7 +4525,7 @@
         </is>
       </c>
     </row>
-    <row r="5">
+    <row r="5" ht="126" customHeight="1">
       <c r="A5" s="2" t="inlineStr">
         <is>
           <t>One beast per army</t>
@@ -4538,12 +4538,12 @@
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>An army never has two beasts, custom armies included.</t>
+          <t>Each army starts with at most one Beast. Morph cannot create a Beast while that side has one. Salvation or Sacrifice may return a captured Beast even if that gives the side a second Beast.</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>Owner 2026-10-04.</t>
+          <t>Owner 2026-10-04: no second Beast. Owner 2026-10-09: a second Beast may return through Salvation or Sacrifice.</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
@@ -4876,7 +4876,7 @@
         </is>
       </c>
     </row>
-    <row r="18">
+    <row r="18" ht="78" customHeight="1">
       <c r="A18" s="2" t="inlineStr">
         <is>
           <t>Hand size</t>
@@ -4889,12 +4889,12 @@
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>Six cards a side.</t>
+          <t>Four starting cards per side.</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>Owner 2026-10-03: six. Owner 2026-10-08: more cards means fewer draws; the question is closed. Draws at d4: none 29.7%, 2 cards 17.5, 3 15.5, 4 12.6, 6 11.0.</t>
+          <t>Owner 2026-10-03: six. Owner 2026-10-08: more cards means fewer draws; the question is closed. Draws at d4: none 29.7%, 2 cards 17.5, 3 15.5, 4 12.6, 6 11.0. Owner 2026-10-09: four starting cards.</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
@@ -4916,7 +4916,7 @@
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>The cards the six are dealt from.</t>
+          <t>The cards the starting hand is dealt from.</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">

</xml_diff>